<commit_message>
Add stress (0.0880) to nmds_results.xlsx Metadata
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nmds_results.xlsx
+++ b/nmds_results.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card_WA_Scores" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6988,4 +6989,30 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>stress</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0.08799999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>